<commit_message>
(PROBLEM SEND MAIL) feat: implement notification workflows for secretary alerts and patient appointment confirmations
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -87,9 +87,6 @@
     <t>SmtpServer</t>
   </si>
   <si>
-    <t>smtp.example.com</t>
-  </si>
-  <si>
     <t>Serveur SMTP</t>
   </si>
   <si>
@@ -147,10 +144,13 @@
     <t>Cabinet Médical Dr. Mahdi</t>
   </si>
   <si>
-    <t>toew ipog fyop rvnk</t>
-  </si>
-  <si>
     <t>mahdilaith08@gmail.com</t>
+  </si>
+  <si>
+    <t>smtp.gmail.com</t>
+  </si>
+  <si>
+    <t>toewipogfyoprvnk</t>
   </si>
 </sst>
 </file>
@@ -623,7 +623,7 @@
         <v>15</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>16</v>
@@ -634,7 +634,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>18</v>
@@ -645,7 +645,7 @@
         <v>19</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>20</v>
@@ -656,76 +656,76 @@
         <v>21</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13" s="3">
         <v>21653843799</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement patient notification and secretary notification workflows with supporting configuration and log files
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -141,16 +141,16 @@
     <t>loussaiefdalel15@gmail.com</t>
   </si>
   <si>
-    <t>Cabinet Médical Dr. Mahdi</t>
-  </si>
-  <si>
     <t>mahdilaith08@gmail.com</t>
   </si>
   <si>
     <t>smtp.gmail.com</t>
   </si>
   <si>
-    <t>toewipogfyoprvnk</t>
+    <t>lziu ikmw cvks thja</t>
+  </si>
+  <si>
+    <t>Cabinet Médical Dr. Mahdi Laith</t>
   </si>
 </sst>
 </file>
@@ -634,7 +634,7 @@
         <v>17</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>18</v>
@@ -645,7 +645,7 @@
         <v>19</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>20</v>
@@ -656,7 +656,7 @@
         <v>21</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>22</v>
@@ -678,7 +678,7 @@
         <v>26</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>27</v>
@@ -689,7 +689,7 @@
         <v>28</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>29</v>

</xml_diff>